<commit_message>
Adicionando dicionário de dados com descrição
</commit_message>
<xml_diff>
--- a/Book/Sprint 2/DicionarioDeDados/DicionarioDeDadosV2.xlsx
+++ b/Book/Sprint 2/DicionarioDeDados/DicionarioDeDadosV2.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marquinhos\Desktop\sptech\2025\2 Semestre\PI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User.DESKTOP-28VA7A5\Desktop\Sptech\2025\2ºSemestre\Sprint 03\PI\TEP\Book\Sprint 2\DicionarioDeDados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FD22A030-A3FE-4D41-9FF9-254668891BD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13740" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13740" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="coloque tudo em uma mesma tabel" sheetId="1" r:id="rId1"/>
@@ -21,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="108">
   <si>
     <t>Tabela</t>
   </si>
@@ -323,12 +322,37 @@
   </si>
   <si>
     <t>E-mail de contato da empresa.</t>
+  </si>
+  <si>
+    <t>Armazena as informações sobre as regiões geográficas, incluindo o nome completo e a sigla identificadora de cada uma.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guarda os valores de indicadores econômicos (como valor adicionado) de cada setor em um município específico, em determinado ano.
+</t>
+  </si>
+  <si>
+    <t>Registra os diferentes setores de atividade econômica (como indústria, comércio, serviços, etc.), utilizados para classificar os indicadores econômicos.</t>
+  </si>
+  <si>
+    <t>Armazena as informações dos usuários do sistema, incluindo dados de acesso, data de criação e se possuem perfil de administrador.</t>
+  </si>
+  <si>
+    <t>Reúne os dados cadastrais das empresas, como razão social, CNPJ, e informações de contato.</t>
+  </si>
+  <si>
+    <t>Registra as métricas econômicas de cada município em um determinado ano, como impostos arrecadados, PIB total e PIB per capita.</t>
+  </si>
+  <si>
+    <t>Responsável por registrar o histórico de ações realizadas no banco de dados.</t>
+  </si>
+  <si>
+    <t>Contém os dados dos municípios, como o nome e a referência à região à qual pertencem.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -381,7 +405,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="21">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -647,11 +671,71 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -695,16 +779,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -757,24 +832,8 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -799,6 +858,99 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1019,7 +1171,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -1057,7 +1209,7 @@
       </c>
     </row>
     <row r="3" spans="2:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="47" t="s">
         <v>4</v>
       </c>
       <c r="C3" s="1" t="s">
@@ -1075,7 +1227,7 @@
       </c>
     </row>
     <row r="4" spans="2:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="17"/>
+      <c r="B4" s="47"/>
       <c r="C4" s="1" t="s">
         <v>8</v>
       </c>
@@ -1093,7 +1245,7 @@
       </c>
     </row>
     <row r="5" spans="2:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="17"/>
+      <c r="B5" s="47"/>
       <c r="C5" s="1" t="s">
         <v>9</v>
       </c>
@@ -1111,15 +1263,15 @@
       </c>
     </row>
     <row r="6" spans="2:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="17"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="20"/>
+      <c r="B6" s="47"/>
+      <c r="C6" s="49"/>
+      <c r="D6" s="49"/>
+      <c r="E6" s="49"/>
+      <c r="F6" s="49"/>
+      <c r="G6" s="50"/>
     </row>
     <row r="7" spans="2:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="47" t="s">
         <v>10</v>
       </c>
       <c r="C7" s="1" t="s">
@@ -1137,7 +1289,7 @@
       </c>
     </row>
     <row r="8" spans="2:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="17"/>
+      <c r="B8" s="47"/>
       <c r="C8" s="1" t="s">
         <v>13</v>
       </c>
@@ -1155,7 +1307,7 @@
       </c>
     </row>
     <row r="9" spans="2:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="17"/>
+      <c r="B9" s="47"/>
       <c r="C9" s="1" t="s">
         <v>15</v>
       </c>
@@ -1171,15 +1323,15 @@
       </c>
     </row>
     <row r="10" spans="2:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="17"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="20"/>
+      <c r="B10" s="47"/>
+      <c r="C10" s="49"/>
+      <c r="D10" s="49"/>
+      <c r="E10" s="49"/>
+      <c r="F10" s="49"/>
+      <c r="G10" s="50"/>
     </row>
     <row r="11" spans="2:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="47" t="s">
         <v>17</v>
       </c>
       <c r="C11" s="1" t="s">
@@ -1197,7 +1349,7 @@
       </c>
     </row>
     <row r="12" spans="2:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="17"/>
+      <c r="B12" s="47"/>
       <c r="C12" s="1" t="s">
         <v>19</v>
       </c>
@@ -1215,15 +1367,15 @@
       </c>
     </row>
     <row r="13" spans="2:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="17"/>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
-      <c r="G13" s="20"/>
+      <c r="B13" s="47"/>
+      <c r="C13" s="49"/>
+      <c r="D13" s="49"/>
+      <c r="E13" s="49"/>
+      <c r="F13" s="49"/>
+      <c r="G13" s="50"/>
     </row>
     <row r="14" spans="2:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="47" t="s">
         <v>21</v>
       </c>
       <c r="C14" s="1" t="s">
@@ -1241,7 +1393,7 @@
       </c>
     </row>
     <row r="15" spans="2:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="17"/>
+      <c r="B15" s="47"/>
       <c r="C15" s="1" t="s">
         <v>24</v>
       </c>
@@ -1257,7 +1409,7 @@
       </c>
     </row>
     <row r="16" spans="2:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="17"/>
+      <c r="B16" s="47"/>
       <c r="C16" s="1" t="s">
         <v>27</v>
       </c>
@@ -1275,7 +1427,7 @@
       </c>
     </row>
     <row r="17" spans="2:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="17"/>
+      <c r="B17" s="47"/>
       <c r="C17" s="1" t="s">
         <v>28</v>
       </c>
@@ -1293,7 +1445,7 @@
       </c>
     </row>
     <row r="18" spans="2:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="17"/>
+      <c r="B18" s="47"/>
       <c r="C18" s="1" t="s">
         <v>30</v>
       </c>
@@ -1311,7 +1463,7 @@
       </c>
     </row>
     <row r="19" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="17"/>
+      <c r="B19" s="47"/>
       <c r="C19" s="1" t="s">
         <v>32</v>
       </c>
@@ -1327,7 +1479,7 @@
       </c>
     </row>
     <row r="20" spans="2:7" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="18"/>
+      <c r="B20" s="48"/>
       <c r="C20" s="11" t="s">
         <v>33</v>
       </c>
@@ -1361,824 +1513,988 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED9847B3-073E-4A5D-B67E-1A37C2748D6A}">
-  <dimension ref="B1:I47"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K49"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.5703125" style="24" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16" style="22" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5703125" style="22" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="34" style="21" customWidth="1"/>
-    <col min="8" max="8" width="71.42578125" style="28" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.85546875" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.5703125" style="21" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16" style="19" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.5703125" style="19" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="34" style="18" customWidth="1"/>
+    <col min="10" max="10" width="71.42578125" style="25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:8" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:8" s="23" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="B2" s="44"/>
-      <c r="C2" s="38" t="s">
+    <row r="1" spans="1:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:10" s="20" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="A2" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="26" t="s">
+      <c r="F2" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="G2" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="H2" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="G2" s="15" t="s">
+      <c r="I2" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="H2" s="29" t="s">
+      <c r="J2" s="26" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B3" s="45"/>
-      <c r="C3" s="39" t="s">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" s="66" t="s">
+        <v>100</v>
+      </c>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="25" t="s">
+      <c r="F3" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="G3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4" t="s">
+      <c r="H3" s="4"/>
+      <c r="I3" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="H3" s="27" t="s">
+      <c r="J3" s="24" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B4" s="45"/>
-      <c r="C4" s="39"/>
-      <c r="D4" s="25" t="s">
+    <row r="4" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="61"/>
+      <c r="B4" s="56"/>
+      <c r="C4" s="56"/>
+      <c r="D4" s="62"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="F4" s="4">
-        <v>45</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="H4" s="27" t="s">
+      <c r="H4" s="4">
+        <v>45</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="J4" s="24" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B5" s="45"/>
-      <c r="C5" s="39"/>
-      <c r="D5" s="25" t="s">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5" s="63"/>
+      <c r="B5" s="64"/>
+      <c r="C5" s="64"/>
+      <c r="D5" s="65"/>
+      <c r="E5" s="55"/>
+      <c r="F5" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="G5" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="F5" s="4">
+      <c r="H5" s="4">
         <v>2</v>
       </c>
-      <c r="G5" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="H5" s="27" t="s">
+      <c r="I5" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="J5" s="24" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B6" s="45"/>
-      <c r="C6" s="39"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="19"/>
-      <c r="H6" s="20"/>
-    </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B7" s="45"/>
-      <c r="C7" s="39" t="s">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="D6" s="37"/>
+      <c r="E6" s="55"/>
+      <c r="F6" s="49"/>
+      <c r="G6" s="49"/>
+      <c r="H6" s="49"/>
+      <c r="I6" s="49"/>
+      <c r="J6" s="50"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" s="68" t="s">
+        <v>107</v>
+      </c>
+      <c r="B7" s="69"/>
+      <c r="C7" s="69"/>
+      <c r="D7" s="70"/>
+      <c r="E7" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="25" t="s">
+      <c r="F7" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="G7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4" t="s">
+      <c r="H7" s="4"/>
+      <c r="I7" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="H7" s="27" t="s">
+      <c r="J7" s="24" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B8" s="45"/>
-      <c r="C8" s="39"/>
-      <c r="D8" s="25" t="s">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A8" s="71"/>
+      <c r="B8" s="72"/>
+      <c r="C8" s="72"/>
+      <c r="D8" s="73"/>
+      <c r="E8" s="55"/>
+      <c r="F8" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="G8" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="F8" s="4">
-        <v>45</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="H8" s="27" t="s">
+      <c r="H8" s="4">
+        <v>45</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="J8" s="24" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="2:8" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="B9" s="45"/>
-      <c r="C9" s="39"/>
-      <c r="D9" s="25" t="s">
+    <row r="9" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A9" s="74"/>
+      <c r="B9" s="75"/>
+      <c r="C9" s="75"/>
+      <c r="D9" s="76"/>
+      <c r="E9" s="55"/>
+      <c r="F9" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="G9" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="H9" s="27" t="s">
+      <c r="H9" s="4"/>
+      <c r="I9" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="J9" s="24" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B10" s="45"/>
-      <c r="C10" s="39"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="19"/>
-      <c r="H10" s="20"/>
-    </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B11" s="45"/>
-      <c r="C11" s="39" t="s">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="D10" s="37"/>
+      <c r="E10" s="55"/>
+      <c r="F10" s="49"/>
+      <c r="G10" s="49"/>
+      <c r="H10" s="49"/>
+      <c r="I10" s="49"/>
+      <c r="J10" s="50"/>
+    </row>
+    <row r="11" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="66" t="s">
+        <v>102</v>
+      </c>
+      <c r="B11" s="59"/>
+      <c r="C11" s="59"/>
+      <c r="D11" s="60"/>
+      <c r="E11" s="53" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="25" t="s">
+      <c r="F11" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="G11" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4" t="s">
+      <c r="H11" s="4"/>
+      <c r="I11" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="H11" s="27" t="s">
+      <c r="J11" s="24" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B12" s="45"/>
-      <c r="C12" s="39"/>
-      <c r="D12" s="25" t="s">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A12" s="61"/>
+      <c r="B12" s="56"/>
+      <c r="C12" s="56"/>
+      <c r="D12" s="62"/>
+      <c r="E12" s="54"/>
+      <c r="F12" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="G12" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="F12" s="4">
-        <v>45</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="H12" s="27" t="s">
+      <c r="H12" s="4">
+        <v>45</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="J12" s="24" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B13" s="45"/>
-      <c r="C13" s="39"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
-      <c r="G13" s="19"/>
-      <c r="H13" s="20"/>
-    </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B14" s="45"/>
-      <c r="C14" s="40" t="s">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A13" s="61"/>
+      <c r="B13" s="56"/>
+      <c r="C13" s="56"/>
+      <c r="D13" s="62"/>
+      <c r="E13" s="54"/>
+      <c r="F13" s="22"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="17"/>
+      <c r="J13" s="24"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A14" s="63"/>
+      <c r="B14" s="64"/>
+      <c r="C14" s="64"/>
+      <c r="D14" s="65"/>
+      <c r="E14" s="67"/>
+      <c r="F14" s="22"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="17"/>
+      <c r="J14" s="24"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="D15" s="37"/>
+      <c r="E15" s="55"/>
+      <c r="F15" s="49"/>
+      <c r="G15" s="49"/>
+      <c r="H15" s="49"/>
+      <c r="I15" s="49"/>
+      <c r="J15" s="50"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A16" s="77" t="s">
+        <v>101</v>
+      </c>
+      <c r="B16" s="69"/>
+      <c r="C16" s="69"/>
+      <c r="D16" s="70"/>
+      <c r="E16" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="D14" s="25" t="s">
+      <c r="F16" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="G16" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4" t="s">
+      <c r="H16" s="4"/>
+      <c r="I16" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="H14" s="27" t="s">
+      <c r="J16" s="24" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B15" s="45"/>
-      <c r="C15" s="41"/>
-      <c r="D15" s="25" t="s">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A17" s="71"/>
+      <c r="B17" s="72"/>
+      <c r="C17" s="72"/>
+      <c r="D17" s="73"/>
+      <c r="E17" s="54"/>
+      <c r="F17" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="G17" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="H15" s="27" t="s">
+      <c r="H17" s="4"/>
+      <c r="I17" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="J17" s="24" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B16" s="45"/>
-      <c r="C16" s="41"/>
-      <c r="D16" s="25" t="s">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A18" s="71"/>
+      <c r="B18" s="72"/>
+      <c r="C18" s="72"/>
+      <c r="D18" s="73"/>
+      <c r="E18" s="54"/>
+      <c r="F18" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="G18" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="F16" s="4">
+      <c r="H18" s="4">
         <v>18.2</v>
       </c>
-      <c r="G16" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="H16" s="27" t="s">
+      <c r="I18" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="J18" s="24" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="17" spans="2:9" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="B17" s="45"/>
-      <c r="C17" s="41"/>
-      <c r="D17" s="25" t="s">
+    <row r="19" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A19" s="71"/>
+      <c r="B19" s="72"/>
+      <c r="C19" s="72"/>
+      <c r="D19" s="73"/>
+      <c r="E19" s="54"/>
+      <c r="F19" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="G19" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4" t="s">
+      <c r="H19" s="4"/>
+      <c r="I19" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="H17" s="27" t="s">
+      <c r="J19" s="24" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="18" spans="2:9" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="B18" s="45"/>
-      <c r="C18" s="41"/>
-      <c r="D18" s="30" t="s">
+    <row r="20" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A20" s="74"/>
+      <c r="B20" s="75"/>
+      <c r="C20" s="75"/>
+      <c r="D20" s="76"/>
+      <c r="E20" s="54"/>
+      <c r="F20" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="E18" s="31" t="s">
+      <c r="G20" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="F18" s="31"/>
-      <c r="G18" s="31" t="s">
+      <c r="H20" s="28"/>
+      <c r="I20" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="H18" s="32" t="s">
+      <c r="J20" s="29" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="45"/>
-      <c r="C19" s="42"/>
-      <c r="D19" s="33"/>
-      <c r="E19" s="34"/>
-      <c r="F19" s="34"/>
-      <c r="G19" s="34"/>
-      <c r="H19" s="54"/>
-      <c r="I19" s="37"/>
-    </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="45"/>
-      <c r="C20" s="43" t="s">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="D21" s="37"/>
+      <c r="E21" s="36"/>
+      <c r="F21" s="30"/>
+      <c r="G21" s="31"/>
+      <c r="H21" s="31"/>
+      <c r="I21" s="31"/>
+      <c r="J21" s="45"/>
+      <c r="K21" s="34"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A22" s="77" t="s">
+        <v>103</v>
+      </c>
+      <c r="B22" s="69"/>
+      <c r="C22" s="69"/>
+      <c r="D22" s="70"/>
+      <c r="E22" s="51" t="s">
         <v>48</v>
       </c>
-      <c r="D20" s="35" t="s">
+      <c r="F22" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="E20" s="36" t="s">
+      <c r="G22" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="F20" s="36"/>
-      <c r="G20" s="36" t="s">
+      <c r="H22" s="33"/>
+      <c r="I22" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="H20" s="54" t="s">
+      <c r="J22" s="45" t="s">
         <v>75</v>
       </c>
-      <c r="I20" s="37"/>
-    </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B21" s="45"/>
-      <c r="C21" s="43"/>
-      <c r="D21" s="35" t="s">
+      <c r="K22" s="34"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A23" s="71"/>
+      <c r="B23" s="72"/>
+      <c r="C23" s="72"/>
+      <c r="D23" s="73"/>
+      <c r="E23" s="51"/>
+      <c r="F23" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="E21" s="36" t="s">
+      <c r="G23" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="F21" s="36">
+      <c r="H23" s="33">
         <v>60</v>
       </c>
-      <c r="G21" s="36" t="s">
-        <v>45</v>
-      </c>
-      <c r="H21" s="54" t="s">
+      <c r="I23" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="J23" s="45" t="s">
         <v>76</v>
       </c>
-      <c r="I21" s="37"/>
-    </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B22" s="45"/>
-      <c r="C22" s="43"/>
-      <c r="D22" s="35" t="s">
+      <c r="K23" s="34"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A24" s="71"/>
+      <c r="B24" s="72"/>
+      <c r="C24" s="72"/>
+      <c r="D24" s="73"/>
+      <c r="E24" s="51"/>
+      <c r="F24" s="32" t="s">
         <v>51</v>
       </c>
-      <c r="E22" s="36" t="s">
+      <c r="G24" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="F22" s="36">
+      <c r="H24" s="33">
         <v>100</v>
       </c>
-      <c r="G22" s="36" t="s">
-        <v>45</v>
-      </c>
-      <c r="H22" s="54" t="s">
+      <c r="I24" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="J24" s="45" t="s">
         <v>77</v>
       </c>
-      <c r="I22" s="37"/>
-    </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B23" s="45"/>
-      <c r="C23" s="43"/>
-      <c r="D23" s="35" t="s">
+      <c r="K24" s="34"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A25" s="71"/>
+      <c r="B25" s="72"/>
+      <c r="C25" s="72"/>
+      <c r="D25" s="73"/>
+      <c r="E25" s="51"/>
+      <c r="F25" s="32" t="s">
         <v>52</v>
       </c>
-      <c r="E23" s="36" t="s">
+      <c r="G25" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="F23" s="36">
+      <c r="H25" s="33">
         <v>100</v>
       </c>
-      <c r="G23" s="36" t="s">
-        <v>45</v>
-      </c>
-      <c r="H23" s="54" t="s">
+      <c r="I25" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="J25" s="45" t="s">
         <v>97</v>
       </c>
-      <c r="I23" s="37"/>
-    </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B24" s="45"/>
-      <c r="C24" s="43"/>
-      <c r="D24" s="35" t="s">
+      <c r="K25" s="34"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A26" s="71"/>
+      <c r="B26" s="72"/>
+      <c r="C26" s="72"/>
+      <c r="D26" s="73"/>
+      <c r="E26" s="51"/>
+      <c r="F26" s="32" t="s">
         <v>53</v>
       </c>
-      <c r="E24" s="36" t="s">
+      <c r="G26" s="33" t="s">
         <v>54</v>
       </c>
-      <c r="F24" s="36"/>
-      <c r="G24" s="36" t="s">
+      <c r="H26" s="33"/>
+      <c r="I26" s="33" t="s">
         <v>55</v>
       </c>
-      <c r="H24" s="54" t="s">
+      <c r="J26" s="45" t="s">
         <v>78</v>
       </c>
-      <c r="I24" s="37"/>
-    </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B25" s="45"/>
-      <c r="C25" s="43"/>
-      <c r="D25" s="35" t="s">
+      <c r="K26" s="34"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A27" s="71"/>
+      <c r="B27" s="72"/>
+      <c r="C27" s="72"/>
+      <c r="D27" s="73"/>
+      <c r="E27" s="51"/>
+      <c r="F27" s="32" t="s">
         <v>56</v>
       </c>
-      <c r="E25" s="36" t="s">
+      <c r="G27" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="F25" s="36"/>
-      <c r="G25" s="36" t="s">
+      <c r="H27" s="33"/>
+      <c r="I27" s="33" t="s">
         <v>46</v>
       </c>
-      <c r="H25" s="54" t="s">
+      <c r="J27" s="45" t="s">
         <v>79</v>
       </c>
-      <c r="I25" s="37"/>
-    </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B26" s="45"/>
-      <c r="C26" s="43"/>
-      <c r="D26" s="35" t="s">
+      <c r="K27" s="34"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A28" s="74"/>
+      <c r="B28" s="75"/>
+      <c r="C28" s="75"/>
+      <c r="D28" s="76"/>
+      <c r="E28" s="51"/>
+      <c r="F28" s="32" t="s">
         <v>57</v>
       </c>
-      <c r="E26" s="36" t="s">
+      <c r="G28" s="33" t="s">
         <v>58</v>
       </c>
-      <c r="F26" s="36"/>
-      <c r="G26" s="36" t="s">
+      <c r="H28" s="33"/>
+      <c r="I28" s="33" t="s">
         <v>59</v>
       </c>
-      <c r="H26" s="54" t="s">
+      <c r="J28" s="45" t="s">
         <v>96</v>
       </c>
-      <c r="I26" s="37"/>
-    </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B27" s="45"/>
-      <c r="C27" s="42"/>
-      <c r="D27" s="33"/>
-      <c r="E27" s="34"/>
-      <c r="F27" s="34"/>
-      <c r="G27" s="34"/>
-      <c r="H27" s="54"/>
-      <c r="I27" s="37"/>
-    </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B28" s="45"/>
-      <c r="C28" s="43" t="s">
+      <c r="K28" s="34"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="D29" s="37"/>
+      <c r="E29" s="36"/>
+      <c r="F29" s="30"/>
+      <c r="G29" s="31"/>
+      <c r="H29" s="31"/>
+      <c r="I29" s="31"/>
+      <c r="J29" s="45"/>
+      <c r="K29" s="34"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A30" s="77" t="s">
+        <v>104</v>
+      </c>
+      <c r="B30" s="69"/>
+      <c r="C30" s="69"/>
+      <c r="D30" s="70"/>
+      <c r="E30" s="51" t="s">
         <v>60</v>
       </c>
-      <c r="D28" s="35" t="s">
+      <c r="F30" s="32" t="s">
         <v>61</v>
       </c>
-      <c r="E28" s="36" t="s">
+      <c r="G30" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="F28" s="36"/>
-      <c r="G28" s="36" t="s">
+      <c r="H30" s="33"/>
+      <c r="I30" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="H28" s="54" t="s">
+      <c r="J30" s="45" t="s">
         <v>80</v>
       </c>
-      <c r="I28" s="37"/>
-    </row>
-    <row r="29" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B29" s="45"/>
-      <c r="C29" s="43"/>
-      <c r="D29" s="35" t="s">
+      <c r="K30" s="34"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A31" s="71"/>
+      <c r="B31" s="72"/>
+      <c r="C31" s="72"/>
+      <c r="D31" s="73"/>
+      <c r="E31" s="51"/>
+      <c r="F31" s="32" t="s">
         <v>62</v>
       </c>
-      <c r="E29" s="36" t="s">
+      <c r="G31" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="F29" s="36">
+      <c r="H31" s="33">
         <v>100</v>
       </c>
-      <c r="G29" s="36" t="s">
-        <v>45</v>
-      </c>
-      <c r="H29" s="54" t="s">
+      <c r="I31" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="J31" s="45" t="s">
         <v>81</v>
       </c>
-      <c r="I29" s="37"/>
-    </row>
-    <row r="30" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B30" s="45"/>
-      <c r="C30" s="43"/>
-      <c r="D30" s="35" t="s">
+      <c r="K31" s="34"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A32" s="71"/>
+      <c r="B32" s="72"/>
+      <c r="C32" s="72"/>
+      <c r="D32" s="73"/>
+      <c r="E32" s="51"/>
+      <c r="F32" s="32" t="s">
         <v>63</v>
       </c>
-      <c r="E30" s="36" t="s">
+      <c r="G32" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="F30" s="36">
+      <c r="H32" s="33">
         <v>14</v>
       </c>
-      <c r="G30" s="36" t="s">
+      <c r="I32" s="33" t="s">
         <v>64</v>
       </c>
-      <c r="H30" s="54" t="s">
+      <c r="J32" s="45" t="s">
         <v>98</v>
       </c>
-      <c r="I30" s="37"/>
-    </row>
-    <row r="31" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B31" s="45"/>
-      <c r="C31" s="43"/>
-      <c r="D31" s="35" t="s">
+      <c r="K32" s="34"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A33" s="71"/>
+      <c r="B33" s="72"/>
+      <c r="C33" s="72"/>
+      <c r="D33" s="73"/>
+      <c r="E33" s="51"/>
+      <c r="F33" s="32" t="s">
         <v>51</v>
       </c>
-      <c r="E31" s="36" t="s">
+      <c r="G33" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="F31" s="36">
+      <c r="H33" s="33">
         <v>100</v>
       </c>
-      <c r="G31" s="36" t="s">
-        <v>45</v>
-      </c>
-      <c r="H31" s="54" t="s">
+      <c r="I33" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="J33" s="45" t="s">
         <v>99</v>
       </c>
-      <c r="I31" s="37"/>
-    </row>
-    <row r="32" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B32" s="45"/>
-      <c r="C32" s="43"/>
-      <c r="D32" s="35" t="s">
+      <c r="K33" s="34"/>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A34" s="71"/>
+      <c r="B34" s="72"/>
+      <c r="C34" s="72"/>
+      <c r="D34" s="73"/>
+      <c r="E34" s="51"/>
+      <c r="F34" s="32" t="s">
         <v>52</v>
       </c>
-      <c r="E32" s="36" t="s">
+      <c r="G34" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="F32" s="36">
+      <c r="H34" s="33">
         <v>100</v>
       </c>
-      <c r="G32" s="36" t="s">
-        <v>45</v>
-      </c>
-      <c r="H32" s="54" t="s">
+      <c r="I34" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="J34" s="45" t="s">
         <v>82</v>
       </c>
-      <c r="I32" s="37"/>
-    </row>
-    <row r="33" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B33" s="45"/>
-      <c r="C33" s="43"/>
-      <c r="D33" s="35" t="s">
+      <c r="K34" s="34"/>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A35" s="74"/>
+      <c r="B35" s="75"/>
+      <c r="C35" s="75"/>
+      <c r="D35" s="76"/>
+      <c r="E35" s="51"/>
+      <c r="F35" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="E33" s="36" t="s">
+      <c r="G35" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="F33" s="36"/>
-      <c r="G33" s="36" t="s">
+      <c r="H35" s="33"/>
+      <c r="I35" s="33" t="s">
         <v>46</v>
       </c>
-      <c r="H33" s="54" t="s">
+      <c r="J35" s="45" t="s">
         <v>83</v>
       </c>
-      <c r="I33" s="37"/>
-    </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B34" s="45"/>
-      <c r="C34" s="42"/>
-      <c r="D34" s="33"/>
-      <c r="E34" s="34"/>
-      <c r="F34" s="34"/>
-      <c r="G34" s="34"/>
-      <c r="H34" s="54"/>
-      <c r="I34" s="37"/>
-    </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B35" s="45"/>
-      <c r="C35" s="42"/>
-      <c r="D35" s="33"/>
-      <c r="E35" s="34"/>
-      <c r="F35" s="34"/>
-      <c r="G35" s="34"/>
-      <c r="H35" s="54"/>
-      <c r="I35" s="37"/>
-    </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B36" s="45"/>
-      <c r="C36" s="43" t="s">
+      <c r="K35" s="34"/>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="D36" s="37"/>
+      <c r="E36" s="36"/>
+      <c r="F36" s="30"/>
+      <c r="G36" s="31"/>
+      <c r="H36" s="31"/>
+      <c r="I36" s="31"/>
+      <c r="J36" s="45"/>
+      <c r="K36" s="34"/>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="D37" s="37"/>
+      <c r="E37" s="36"/>
+      <c r="F37" s="30"/>
+      <c r="G37" s="31"/>
+      <c r="H37" s="31"/>
+      <c r="I37" s="31"/>
+      <c r="J37" s="45"/>
+      <c r="K37" s="34"/>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A38" s="77" t="s">
+        <v>105</v>
+      </c>
+      <c r="B38" s="69"/>
+      <c r="C38" s="69"/>
+      <c r="D38" s="70"/>
+      <c r="E38" s="51" t="s">
         <v>65</v>
       </c>
-      <c r="D36" s="35" t="s">
+      <c r="F38" s="32" t="s">
         <v>66</v>
       </c>
-      <c r="E36" s="36" t="s">
+      <c r="G38" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="F36" s="36"/>
-      <c r="G36" s="36" t="s">
+      <c r="H38" s="33"/>
+      <c r="I38" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="H36" s="54" t="s">
+      <c r="J38" s="45" t="s">
         <v>84</v>
       </c>
-      <c r="I36" s="37"/>
-    </row>
-    <row r="37" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B37" s="45"/>
-      <c r="C37" s="43"/>
-      <c r="D37" s="35" t="s">
+      <c r="K38" s="34"/>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A39" s="71"/>
+      <c r="B39" s="72"/>
+      <c r="C39" s="72"/>
+      <c r="D39" s="73"/>
+      <c r="E39" s="51"/>
+      <c r="F39" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="E37" s="36" t="s">
+      <c r="G39" s="33" t="s">
         <v>41</v>
       </c>
-      <c r="F37" s="36">
+      <c r="H39" s="33">
         <v>18.2</v>
       </c>
-      <c r="G37" s="36" t="s">
-        <v>45</v>
-      </c>
-      <c r="H37" s="54" t="s">
+      <c r="I39" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="J39" s="45" t="s">
         <v>85</v>
       </c>
-      <c r="I37" s="37"/>
-    </row>
-    <row r="38" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B38" s="45"/>
-      <c r="C38" s="43"/>
-      <c r="D38" s="35" t="s">
+      <c r="K39" s="34"/>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A40" s="71"/>
+      <c r="B40" s="72"/>
+      <c r="C40" s="72"/>
+      <c r="D40" s="73"/>
+      <c r="E40" s="51"/>
+      <c r="F40" s="32" t="s">
         <v>68</v>
       </c>
-      <c r="E38" s="36" t="s">
+      <c r="G40" s="33" t="s">
         <v>41</v>
       </c>
-      <c r="F38" s="36">
+      <c r="H40" s="33">
         <v>18.2</v>
       </c>
-      <c r="G38" s="36" t="s">
-        <v>45</v>
-      </c>
-      <c r="H38" s="54" t="s">
+      <c r="I40" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="J40" s="45" t="s">
         <v>86</v>
       </c>
-      <c r="I38" s="37"/>
-    </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B39" s="45"/>
-      <c r="C39" s="43"/>
-      <c r="D39" s="35" t="s">
+      <c r="K40" s="34"/>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A41" s="71"/>
+      <c r="B41" s="72"/>
+      <c r="C41" s="72"/>
+      <c r="D41" s="73"/>
+      <c r="E41" s="51"/>
+      <c r="F41" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="E39" s="36" t="s">
+      <c r="G41" s="33" t="s">
         <v>41</v>
       </c>
-      <c r="F39" s="36">
+      <c r="H41" s="33">
         <v>18.2</v>
       </c>
-      <c r="G39" s="36" t="s">
-        <v>45</v>
-      </c>
-      <c r="H39" s="54" t="s">
+      <c r="I41" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="J41" s="45" t="s">
         <v>87</v>
       </c>
-      <c r="I39" s="37"/>
-    </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B40" s="45"/>
-      <c r="C40" s="43"/>
-      <c r="D40" s="35" t="s">
+      <c r="K41" s="34"/>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A42" s="71"/>
+      <c r="B42" s="72"/>
+      <c r="C42" s="72"/>
+      <c r="D42" s="73"/>
+      <c r="E42" s="51"/>
+      <c r="F42" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="E40" s="36" t="s">
+      <c r="G42" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="F40" s="36"/>
-      <c r="G40" s="36" t="s">
-        <v>45</v>
-      </c>
-      <c r="H40" s="54" t="s">
+      <c r="H42" s="33"/>
+      <c r="I42" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="J42" s="45" t="s">
         <v>88</v>
       </c>
-      <c r="I40" s="37"/>
-    </row>
-    <row r="41" spans="2:9" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="B41" s="45"/>
-      <c r="C41" s="43"/>
-      <c r="D41" s="35" t="s">
+      <c r="K42" s="34"/>
+    </row>
+    <row r="43" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A43" s="74"/>
+      <c r="B43" s="75"/>
+      <c r="C43" s="75"/>
+      <c r="D43" s="76"/>
+      <c r="E43" s="51"/>
+      <c r="F43" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="E41" s="36" t="s">
+      <c r="G43" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="F41" s="36"/>
-      <c r="G41" s="36" t="s">
+      <c r="H43" s="33"/>
+      <c r="I43" s="33" t="s">
         <v>46</v>
       </c>
-      <c r="H41" s="54" t="s">
+      <c r="J43" s="45" t="s">
         <v>93</v>
       </c>
-      <c r="I41" s="37"/>
-    </row>
-    <row r="42" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B42" s="45"/>
-      <c r="C42" s="42"/>
-      <c r="D42" s="33"/>
-      <c r="E42" s="34"/>
-      <c r="F42" s="34"/>
-      <c r="G42" s="34"/>
-      <c r="H42" s="54"/>
-      <c r="I42" s="37"/>
-    </row>
-    <row r="43" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B43" s="45"/>
-      <c r="C43" s="43" t="s">
+      <c r="K43" s="34"/>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="D44" s="37"/>
+      <c r="E44" s="36"/>
+      <c r="F44" s="30"/>
+      <c r="G44" s="31"/>
+      <c r="H44" s="31"/>
+      <c r="I44" s="31"/>
+      <c r="J44" s="45"/>
+      <c r="K44" s="34"/>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A45" s="77" t="s">
+        <v>106</v>
+      </c>
+      <c r="B45" s="69"/>
+      <c r="C45" s="69"/>
+      <c r="D45" s="70"/>
+      <c r="E45" s="51" t="s">
         <v>69</v>
       </c>
-      <c r="D43" s="35" t="s">
+      <c r="F45" s="32" t="s">
         <v>70</v>
       </c>
-      <c r="E43" s="36" t="s">
+      <c r="G45" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="F43" s="36"/>
-      <c r="G43" s="36" t="s">
+      <c r="H45" s="33"/>
+      <c r="I45" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="H43" s="54" t="s">
+      <c r="J45" s="45" t="s">
         <v>89</v>
       </c>
-      <c r="I43" s="37"/>
-    </row>
-    <row r="44" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B44" s="45"/>
-      <c r="C44" s="43"/>
-      <c r="D44" s="35" t="s">
+      <c r="K45" s="34"/>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A46" s="71"/>
+      <c r="B46" s="72"/>
+      <c r="C46" s="72"/>
+      <c r="D46" s="73"/>
+      <c r="E46" s="51"/>
+      <c r="F46" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="E44" s="36" t="s">
+      <c r="G46" s="33" t="s">
         <v>72</v>
       </c>
-      <c r="F44" s="36"/>
-      <c r="G44" s="36" t="s">
-        <v>45</v>
-      </c>
-      <c r="H44" s="54" t="s">
+      <c r="H46" s="33"/>
+      <c r="I46" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="J46" s="45" t="s">
         <v>90</v>
       </c>
-      <c r="I44" s="37"/>
-    </row>
-    <row r="45" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B45" s="45"/>
-      <c r="C45" s="43"/>
-      <c r="D45" s="35" t="s">
+      <c r="K46" s="34"/>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A47" s="71"/>
+      <c r="B47" s="72"/>
+      <c r="C47" s="72"/>
+      <c r="D47" s="73"/>
+      <c r="E47" s="51"/>
+      <c r="F47" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="E45" s="36" t="s">
+      <c r="G47" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="F45" s="36">
-        <v>45</v>
-      </c>
-      <c r="G45" s="36" t="s">
-        <v>45</v>
-      </c>
-      <c r="H45" s="54" t="s">
+      <c r="H47" s="33">
+        <v>45</v>
+      </c>
+      <c r="I47" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="J47" s="45" t="s">
         <v>91</v>
       </c>
-      <c r="I45" s="37"/>
-    </row>
-    <row r="46" spans="2:9" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="45"/>
-      <c r="C46" s="46"/>
-      <c r="D46" s="47" t="s">
+      <c r="K47" s="34"/>
+    </row>
+    <row r="48" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="74"/>
+      <c r="B48" s="75"/>
+      <c r="C48" s="75"/>
+      <c r="D48" s="76"/>
+      <c r="E48" s="52"/>
+      <c r="F48" s="38" t="s">
         <v>74</v>
       </c>
-      <c r="E46" s="48" t="s">
+      <c r="G48" s="39" t="s">
         <v>40</v>
       </c>
-      <c r="F46" s="48">
+      <c r="H48" s="39">
         <v>100</v>
       </c>
-      <c r="G46" s="48" t="s">
-        <v>45</v>
-      </c>
-      <c r="H46" s="55" t="s">
+      <c r="I48" s="39" t="s">
+        <v>45</v>
+      </c>
+      <c r="J48" s="46" t="s">
         <v>92</v>
       </c>
-      <c r="I46" s="37"/>
-    </row>
-    <row r="47" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="C47" s="49"/>
-      <c r="D47" s="50"/>
-      <c r="E47" s="51"/>
-      <c r="F47" s="51"/>
-      <c r="G47" s="52"/>
-      <c r="H47" s="53"/>
+      <c r="K48" s="34"/>
+    </row>
+    <row r="49" spans="5:10" x14ac:dyDescent="0.2">
+      <c r="E49" s="40"/>
+      <c r="F49" s="41"/>
+      <c r="G49" s="42"/>
+      <c r="H49" s="42"/>
+      <c r="I49" s="43"/>
+      <c r="J49" s="44"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="C43:C46"/>
-    <mergeCell ref="C14:C18"/>
-    <mergeCell ref="C20:C26"/>
-    <mergeCell ref="C28:C33"/>
-    <mergeCell ref="C36:C41"/>
-    <mergeCell ref="C3:C5"/>
-    <mergeCell ref="C6:H6"/>
-    <mergeCell ref="C7:C9"/>
-    <mergeCell ref="C10:H10"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="C13:H13"/>
+  <mergeCells count="20">
+    <mergeCell ref="A16:D20"/>
+    <mergeCell ref="A22:D28"/>
+    <mergeCell ref="A30:D35"/>
+    <mergeCell ref="A38:D43"/>
+    <mergeCell ref="A45:D48"/>
+    <mergeCell ref="E15:J15"/>
+    <mergeCell ref="A3:D5"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A7:D9"/>
+    <mergeCell ref="A11:D14"/>
+    <mergeCell ref="E11:E14"/>
+    <mergeCell ref="E3:E5"/>
+    <mergeCell ref="E6:J6"/>
+    <mergeCell ref="E7:E9"/>
+    <mergeCell ref="E10:J10"/>
+    <mergeCell ref="E45:E48"/>
+    <mergeCell ref="E16:E20"/>
+    <mergeCell ref="E22:E28"/>
+    <mergeCell ref="E30:E35"/>
+    <mergeCell ref="E38:E43"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>